<commit_message>
Compressed proposal PDF links have been updated
</commit_message>
<xml_diff>
--- a/data/Proposals.xlsx
+++ b/data/Proposals.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC5977CC-177A-412E-90F0-7C7853EEE538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\landscapingUOB-api\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3CD7495-9AF3-4E59-80CB-E90A912D02C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
   <si>
     <t>Location type</t>
   </si>
@@ -172,13 +177,16 @@
   </si>
   <si>
     <t>E-Learning Center</t>
+  </si>
+  <si>
+    <t>https://media.githubusercontent.com/media/UOB-landscape/Landscape-Proposals/main/S1A-S1B-S46.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -222,7 +230,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -238,9 +246,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -577,20 +586,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G62"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" customWidth="1"/>
-    <col min="5" max="5" width="46.42578125" customWidth="1"/>
-    <col min="6" max="6" width="101.42578125" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.54296875" customWidth="1"/>
+    <col min="5" max="5" width="46.453125" customWidth="1"/>
+    <col min="6" max="6" width="101.453125" customWidth="1"/>
+    <col min="7" max="7" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="14.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -611,7 +620,7 @@
       </c>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -627,11 +636,11 @@
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="F2" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -651,17 +660,17 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="7" customFormat="1">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="4" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="5" t="s">
@@ -671,7 +680,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -691,87 +700,87 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" s="7" customFormat="1">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>24</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:7" s="7" customFormat="1">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>24</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:7" s="7" customFormat="1">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>31</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="7" customFormat="1">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="7" t="s">
         <v>34</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -784,14 +793,14 @@
       <c r="D10" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>39</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -808,7 +817,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -825,154 +834,154 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="6:6">
+    <row r="17" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="6:6">
+    <row r="18" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="6:6">
+    <row r="19" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="6:6">
+    <row r="20" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="6:6">
+    <row r="21" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F21" s="1"/>
     </row>
-    <row r="22" spans="6:6">
+    <row r="22" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F22" s="1"/>
     </row>
-    <row r="23" spans="6:6">
+    <row r="23" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="6:6">
+    <row r="24" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F24" s="1"/>
     </row>
-    <row r="25" spans="6:6">
+    <row r="25" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F25" s="1"/>
     </row>
-    <row r="26" spans="6:6">
+    <row r="26" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F26" s="1"/>
     </row>
-    <row r="27" spans="6:6">
+    <row r="27" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="6:6">
+    <row r="28" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="6:6">
+    <row r="29" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F29" s="1"/>
     </row>
-    <row r="30" spans="6:6">
+    <row r="30" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F30" s="1"/>
     </row>
-    <row r="31" spans="6:6">
+    <row r="31" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F31" s="1"/>
     </row>
-    <row r="32" spans="6:6">
+    <row r="32" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F32" s="1"/>
     </row>
-    <row r="33" spans="6:6">
+    <row r="33" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F33" s="1"/>
     </row>
-    <row r="34" spans="6:6">
+    <row r="34" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F34" s="1"/>
     </row>
-    <row r="35" spans="6:6">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F35" s="1"/>
     </row>
-    <row r="36" spans="6:6">
+    <row r="36" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F36" s="1"/>
     </row>
-    <row r="37" spans="6:6">
+    <row r="37" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F37" s="1"/>
     </row>
-    <row r="38" spans="6:6">
+    <row r="38" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F38" s="1"/>
     </row>
-    <row r="39" spans="6:6">
+    <row r="39" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F39" s="1"/>
     </row>
-    <row r="40" spans="6:6">
+    <row r="40" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F40" s="1"/>
     </row>
-    <row r="41" spans="6:6">
+    <row r="41" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F41" s="1"/>
     </row>
-    <row r="42" spans="6:6">
+    <row r="42" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F42" s="1"/>
     </row>
-    <row r="43" spans="6:6">
+    <row r="43" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F43" s="1"/>
     </row>
-    <row r="44" spans="6:6">
+    <row r="44" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F44" s="1"/>
     </row>
-    <row r="45" spans="6:6">
+    <row r="45" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F45" s="1"/>
     </row>
-    <row r="46" spans="6:6">
+    <row r="46" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F46" s="1"/>
     </row>
-    <row r="47" spans="6:6">
+    <row r="47" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F47" s="1"/>
     </row>
-    <row r="48" spans="6:6">
+    <row r="48" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F48" s="1"/>
     </row>
-    <row r="49" spans="6:6">
+    <row r="49" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F49" s="1"/>
     </row>
-    <row r="50" spans="6:6">
+    <row r="50" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F50" s="1"/>
     </row>
-    <row r="51" spans="6:6">
+    <row r="51" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F51" s="1"/>
     </row>
-    <row r="52" spans="6:6">
+    <row r="52" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F52" s="1"/>
     </row>
-    <row r="53" spans="6:6">
+    <row r="53" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F53" s="1"/>
     </row>
-    <row r="54" spans="6:6">
+    <row r="54" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F54" s="1"/>
     </row>
-    <row r="55" spans="6:6">
+    <row r="55" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F55" s="1"/>
     </row>
-    <row r="56" spans="6:6">
+    <row r="56" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F56" s="1"/>
     </row>
-    <row r="57" spans="6:6">
+    <row r="57" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F57" s="1"/>
     </row>
-    <row r="58" spans="6:6">
+    <row r="58" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F58" s="1"/>
     </row>
-    <row r="59" spans="6:6">
+    <row r="59" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F59" s="1"/>
     </row>
-    <row r="60" spans="6:6">
+    <row r="60" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F60" s="1"/>
     </row>
-    <row r="61" spans="6:6">
+    <row r="61" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F61" s="1"/>
     </row>
-    <row r="62" spans="6:6">
+    <row r="62" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F62" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Proposal PDF links have been updated to the new repository name
</commit_message>
<xml_diff>
--- a/data/Proposals.xlsx
+++ b/data/Proposals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\landscapingUOB-api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3CD7495-9AF3-4E59-80CB-E90A912D02C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6374EF76-0DFF-49DF-B10A-2D4885974A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -143,9 +143,6 @@
     <t>https://www.youtube.com/embed/KIqGjib7cZ8</t>
   </si>
   <si>
-    <t>https://media.githubusercontent.com/media/UOB-landscape/Indoor-plants-pdf/main/proposals/Behind College of Arts-Native Trees.pdf</t>
-  </si>
-  <si>
     <t>S39</t>
   </si>
   <si>
@@ -180,6 +177,9 @@
   </si>
   <si>
     <t>https://media.githubusercontent.com/media/UOB-landscape/Landscape-Proposals/main/S1A-S1B-S46.pdf</t>
+  </si>
+  <si>
+    <t>https://media.githubusercontent.com/media/UOB-landscape/PDF-files/main/proposals/Behind College of Arts-Native Trees.pdf</t>
   </si>
 </sst>
 </file>
@@ -637,7 +637,7 @@
         <v>10</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
@@ -777,7 +777,7 @@
         <v>34</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
@@ -785,19 +785,19 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" t="s">
         <v>37</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="F10" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -805,16 +805,16 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" t="s">
         <v>42</v>
       </c>
-      <c r="D11" t="s">
+      <c r="F11" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
@@ -822,16 +822,16 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>46</v>
-      </c>
       <c r="D12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>